<commit_message>
Atualizar tabela: acrescentar figuras russas/soviéticas (Gorbatchov, Iéltsin, Putin) com região de nascimento no campo etnia
</commit_message>
<xml_diff>
--- a/Personagens secundárias (tabela).xlsx
+++ b/Personagens secundárias (tabela).xlsx
@@ -53,7 +53,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -90,6 +90,11 @@
         <fgColor rgb="00595959"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007C0A02"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -117,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -139,6 +144,9 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
@@ -506,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -562,7 +570,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Etnia</t>
+          <t>Etnia / Região</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -1175,7 +1183,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Etnia</t>
+          <t>Etnia / Região</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -1304,7 +1312,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Etnia</t>
+          <t>Etnia / Região</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -1720,11 +1728,261 @@
         </is>
       </c>
     </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Figuras russas / soviéticas (contexto da Guerra Fria)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Nome curto</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Nome completo</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Naturalidade</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Etnia / Região</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Nascimento</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Falecimento</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>Idade em 1992</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>Filiação</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>Cargo / função</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>Alcunha(s)</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>Estatuto na trama (1992)</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="42" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Gorbatchov</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Mikhail Sergueievich Gorbatchov</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Privolnoye, Stavropol</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Cáucaso do Norte (região de Stavropol)</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>2 mar 1931</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>30 ago 2022</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>61</v>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>PCUS (Partido Comunista da URSS)</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>Último líder da URSS; secretário-geral do PCUS (1985) e Presidente da URSS (1990–91)</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>«Gorby»</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>Vivo — afastado do poder (URSS dissolvida em dez. 1991)</t>
+        </is>
+      </c>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>Perestroika e Glasnost; Nobel da Paz 1990. Empurrou Moscovo para uma solução negociada em Angola</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="42" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Iéltsin</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Boris Nikolaievich Iéltsin</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Butka, Sverdlovsk</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Urais (região de Sverdlovsk)</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>1 fev 1931</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>23 abr 2007</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>61</v>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>Reformista russo (ex-PCUS)</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>1.º Presidente da Federação Russa (1991–1999)</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>«Tsar Boris», «Batia»</t>
+        </is>
+      </c>
+      <c r="K32" s="6" t="inlineStr">
+        <is>
+          <t>Vivo — Presidente da Rússia</t>
+        </is>
+      </c>
+      <c r="L32" s="6" t="inlineStr">
+        <is>
+          <t>Retirou a Rússia da lógica da Guerra Fria; fim do apoio soviético maciço ao MPLA</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Putin</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Vladimir Vladimirovich Putin</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Leninegrado (São Petersburgo)</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Noroeste da Rússia (Leninegrado)</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>7 out 1952</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>Ex-KGB / independente</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>Oficial da KGB; em 1992, quadro da câmara de São Petersburgo; futuro Presidente da Rússia (2000)</t>
+        </is>
+      </c>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>«Volodya», «Vova», «Tsar Putin»</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>Vivo — funcionário municipal, ainda desconhecido</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="inlineStr">
+        <is>
+          <t>Viria a recuperar a influência russa em África (defesa, petróleo, diamantes)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A20:L20"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A16:L16"/>
+    <mergeCell ref="A29:L29"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A4:L4"/>
   </mergeCells>

</xml_diff>